<commit_message>
update analysis of crises
</commit_message>
<xml_diff>
--- a/Paper/_statistics/datasets/monthly.xlsx
+++ b/Paper/_statistics/datasets/monthly.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benel\Coding\Python\Paper\_statistics\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03ECA147-534A-4C57-A88A-A1B89F559687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B307C3-2598-465D-B44E-B277590EA76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="overall" sheetId="1" r:id="rId1"/>
@@ -3786,6 +3786,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42F446D8-98FD-41C8-83BA-C036B40B6578}">
   <dimension ref="A1:AF25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="12.88671875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -12946,6 +12949,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D011E1-7849-42FD-BCAE-AB5658923D1D}">
   <dimension ref="A1:AF25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="12" max="12" width="8.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">

</xml_diff>